<commit_message>
feat: add modal for expedition and add also affecter button is not showing
</commit_message>
<xml_diff>
--- a/dummy-content/MARJANE-MALL-EXPORT-DATA.xlsx
+++ b/dummy-content/MARJANE-MALL-EXPORT-DATA.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UNK\Desktop\GoFleet-Enhancer\dummy-content\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User1\Desktop\GoFleet-Enhancer\dummy-content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B429A02-3AE0-457C-8943-853C184D8995}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5A89541-5500-4E93-B3DC-600AABDE9ED1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23250" windowHeight="12450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -88,7 +88,7 @@
     </font>
     <font>
       <sz val="12"/>
-      <color theme="0"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -184,7 +184,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -214,6 +214,7 @@
     <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -228,7 +229,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
-        <color theme="0"/>
+        <color theme="1"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -249,7 +250,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
-        <color theme="0"/>
+        <color theme="1"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -283,7 +284,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
-        <color theme="0"/>
+        <color theme="1"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -318,7 +319,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
-        <color theme="0"/>
+        <color theme="1"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -353,7 +354,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
-        <color theme="0"/>
+        <color theme="1"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -388,7 +389,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
-        <color theme="0"/>
+        <color theme="1"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -423,7 +424,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
-        <color theme="0"/>
+        <color theme="1"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -458,7 +459,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
-        <color theme="0"/>
+        <color theme="1"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -493,7 +494,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
-        <color theme="0"/>
+        <color theme="1"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -528,7 +529,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
-        <color theme="0"/>
+        <color theme="1"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -563,7 +564,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
-        <color theme="0"/>
+        <color theme="1"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -622,72 +623,6 @@
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
     <mruColors>
       <color rgb="FFAEFEFC"/>
       <color rgb="FFFFAFAF"/>
@@ -730,10 +665,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="D8DEE9"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="2E3440"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -988,15 +923,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J194"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J196"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="40.140625" style="1" customWidth="1"/>
-    <col min="2" max="10" width="18.85546875" style="1" customWidth="1"/>
-    <col min="11" max="25" width="18.85546875" customWidth="1"/>
+    <col min="1" max="1" width="40.1796875" style="1" customWidth="1"/>
+    <col min="2" max="10" width="18.81640625" style="1" customWidth="1"/>
+    <col min="11" max="25" width="18.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1028,7 +963,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
       <c r="B2" s="4"/>
       <c r="C2" s="5"/>
@@ -1043,7 +978,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3"/>
       <c r="B3" s="4"/>
       <c r="C3" s="5"/>
@@ -1058,7 +993,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3"/>
       <c r="B4" s="4"/>
       <c r="C4" s="5"/>
@@ -1073,7 +1008,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3"/>
       <c r="B5" s="4"/>
       <c r="C5" s="5"/>
@@ -1088,7 +1023,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3"/>
       <c r="B6" s="4"/>
       <c r="C6" s="5"/>
@@ -1103,7 +1038,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3"/>
       <c r="B7" s="4"/>
       <c r="C7" s="5"/>
@@ -1118,7 +1053,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3"/>
       <c r="B8" s="4"/>
       <c r="C8" s="5"/>
@@ -1133,7 +1068,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
       <c r="C9" s="5"/>
@@ -1148,7 +1083,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
       <c r="C10" s="5"/>
@@ -1163,7 +1098,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3"/>
       <c r="B11" s="4"/>
       <c r="C11" s="5"/>
@@ -1178,7 +1113,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
       <c r="C12" s="5"/>
@@ -1193,7 +1128,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3"/>
       <c r="B13" s="4"/>
       <c r="C13" s="5"/>
@@ -1208,7 +1143,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
       <c r="C14" s="5"/>
@@ -1223,7 +1158,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3"/>
       <c r="B15" s="4"/>
       <c r="C15" s="5"/>
@@ -1238,7 +1173,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3"/>
       <c r="B16" s="4"/>
       <c r="C16" s="5"/>
@@ -1253,7 +1188,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3"/>
       <c r="B17" s="4"/>
       <c r="C17" s="5"/>
@@ -1268,7 +1203,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3"/>
       <c r="B18" s="4"/>
       <c r="C18" s="5"/>
@@ -1283,7 +1218,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3"/>
       <c r="B19" s="4"/>
       <c r="C19" s="5"/>
@@ -1298,7 +1233,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
       <c r="C20" s="5"/>
@@ -1313,7 +1248,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3"/>
       <c r="B21" s="4"/>
       <c r="C21" s="5"/>
@@ -1328,7 +1263,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3"/>
       <c r="B22" s="4"/>
       <c r="C22" s="5"/>
@@ -1343,7 +1278,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3"/>
       <c r="B23" s="4"/>
       <c r="C23" s="5"/>
@@ -1358,7 +1293,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3"/>
       <c r="B24" s="4"/>
       <c r="C24" s="5"/>
@@ -1373,7 +1308,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="3"/>
       <c r="B25" s="4"/>
       <c r="C25" s="5"/>
@@ -1388,7 +1323,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="3"/>
       <c r="B26" s="4"/>
       <c r="C26" s="5"/>
@@ -1403,7 +1338,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="3"/>
       <c r="B27" s="4"/>
       <c r="C27" s="5"/>
@@ -1418,7 +1353,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="3"/>
       <c r="B28" s="4"/>
       <c r="C28" s="5"/>
@@ -1433,7 +1368,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="3"/>
       <c r="B29" s="4"/>
       <c r="C29" s="5"/>
@@ -1448,7 +1383,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="3"/>
       <c r="B30" s="4"/>
       <c r="C30" s="5"/>
@@ -1463,7 +1398,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="3"/>
       <c r="B31" s="4"/>
       <c r="C31" s="5"/>
@@ -1478,7 +1413,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="3"/>
       <c r="B32" s="4"/>
       <c r="C32" s="5"/>
@@ -1493,7 +1428,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="3"/>
       <c r="B33" s="4"/>
       <c r="C33" s="5"/>
@@ -1508,7 +1443,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="3"/>
       <c r="B34" s="4"/>
       <c r="C34" s="5"/>
@@ -1523,7 +1458,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="3"/>
       <c r="B35" s="4"/>
       <c r="C35" s="5"/>
@@ -1538,7 +1473,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="3"/>
       <c r="B36" s="4"/>
       <c r="C36" s="5"/>
@@ -1553,7 +1488,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="3"/>
       <c r="B37" s="4"/>
       <c r="C37" s="5"/>
@@ -1568,7 +1503,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="3"/>
       <c r="B38" s="4"/>
       <c r="C38" s="5"/>
@@ -1583,7 +1518,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="3"/>
       <c r="B39" s="4"/>
       <c r="C39" s="5"/>
@@ -1598,7 +1533,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="3"/>
       <c r="B40" s="4"/>
       <c r="C40" s="5"/>
@@ -1613,7 +1548,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="3"/>
       <c r="B41" s="4"/>
       <c r="C41" s="5"/>
@@ -1628,7 +1563,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="3"/>
       <c r="B42" s="4"/>
       <c r="C42" s="5"/>
@@ -1643,7 +1578,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="3"/>
       <c r="B43" s="4"/>
       <c r="C43" s="5"/>
@@ -1658,7 +1593,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="3"/>
       <c r="B44" s="4"/>
       <c r="C44" s="5"/>
@@ -1673,7 +1608,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="3"/>
       <c r="B45" s="4"/>
       <c r="C45" s="5"/>
@@ -1688,7 +1623,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
       <c r="C46" s="5"/>
@@ -1703,7 +1638,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="3"/>
       <c r="B47" s="4"/>
       <c r="C47" s="5"/>
@@ -1718,7 +1653,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="3"/>
       <c r="B48" s="4"/>
       <c r="C48" s="5"/>
@@ -1733,7 +1668,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="3"/>
       <c r="B49" s="4"/>
       <c r="C49" s="5"/>
@@ -1748,7 +1683,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="3"/>
       <c r="B50" s="4"/>
       <c r="C50" s="5"/>
@@ -1763,7 +1698,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="3"/>
       <c r="B51" s="4"/>
       <c r="C51" s="5"/>
@@ -1778,7 +1713,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="3"/>
       <c r="B52" s="4"/>
       <c r="C52" s="5"/>
@@ -1793,7 +1728,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="3"/>
       <c r="B53" s="4"/>
       <c r="C53" s="5"/>
@@ -1808,7 +1743,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="3"/>
       <c r="B54" s="4"/>
       <c r="C54" s="5"/>
@@ -1823,7 +1758,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="3"/>
       <c r="B55" s="4"/>
       <c r="C55" s="5"/>
@@ -1838,7 +1773,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="3"/>
       <c r="B56" s="4"/>
       <c r="C56" s="5"/>
@@ -1853,7 +1788,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="3"/>
       <c r="B57" s="4"/>
       <c r="C57" s="5"/>
@@ -1868,7 +1803,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="3"/>
       <c r="B58" s="4"/>
       <c r="C58" s="5"/>
@@ -1883,7 +1818,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="3"/>
       <c r="B59" s="4"/>
       <c r="C59" s="5"/>
@@ -1898,7 +1833,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="3"/>
       <c r="B60" s="4"/>
       <c r="C60" s="5"/>
@@ -1913,7 +1848,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="3"/>
       <c r="B61" s="4"/>
       <c r="C61" s="5"/>
@@ -1928,7 +1863,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="3"/>
       <c r="B62" s="4"/>
       <c r="C62" s="5"/>
@@ -1943,7 +1878,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="63" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="3"/>
       <c r="B63" s="4"/>
       <c r="C63" s="5"/>
@@ -1958,7 +1893,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="3"/>
       <c r="B64" s="4"/>
       <c r="C64" s="5"/>
@@ -1973,7 +1908,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="3"/>
       <c r="B65" s="4"/>
       <c r="C65" s="5"/>
@@ -1988,7 +1923,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="3"/>
       <c r="B66" s="4"/>
       <c r="C66" s="5"/>
@@ -2003,7 +1938,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="3"/>
       <c r="B67" s="4"/>
       <c r="C67" s="5"/>
@@ -2018,7 +1953,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="3"/>
       <c r="B68" s="4"/>
       <c r="C68" s="5"/>
@@ -2033,7 +1968,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="3"/>
       <c r="B69" s="4"/>
       <c r="C69" s="5"/>
@@ -2048,7 +1983,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="3"/>
       <c r="B70" s="4"/>
       <c r="C70" s="5"/>
@@ -2063,7 +1998,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="3"/>
       <c r="B71" s="4"/>
       <c r="C71" s="5"/>
@@ -2078,7 +2013,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="72" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="3"/>
       <c r="B72" s="4"/>
       <c r="C72" s="5"/>
@@ -2093,7 +2028,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="73" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="3"/>
       <c r="B73" s="4"/>
       <c r="C73" s="5"/>
@@ -2108,7 +2043,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="74" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="3"/>
       <c r="B74" s="4"/>
       <c r="C74" s="5"/>
@@ -2123,7 +2058,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="75" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="3"/>
       <c r="B75" s="4"/>
       <c r="C75" s="5"/>
@@ -2138,7 +2073,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="76" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="3"/>
       <c r="B76" s="4"/>
       <c r="C76" s="5"/>
@@ -2153,7 +2088,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="77" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="3"/>
       <c r="B77" s="4"/>
       <c r="C77" s="5"/>
@@ -2168,7 +2103,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="78" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="3"/>
       <c r="B78" s="4"/>
       <c r="C78" s="5"/>
@@ -2183,7 +2118,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="79" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="3"/>
       <c r="B79" s="4"/>
       <c r="C79" s="5"/>
@@ -2198,7 +2133,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="80" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="3"/>
       <c r="B80" s="4"/>
       <c r="C80" s="5"/>
@@ -2213,7 +2148,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="81" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="3"/>
       <c r="B81" s="4"/>
       <c r="C81" s="5"/>
@@ -2228,7 +2163,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="82" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="3"/>
       <c r="B82" s="4"/>
       <c r="C82" s="5"/>
@@ -2243,7 +2178,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="83" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="3"/>
       <c r="B83" s="4"/>
       <c r="C83" s="5"/>
@@ -2258,7 +2193,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="84" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="3"/>
       <c r="B84" s="4"/>
       <c r="C84" s="5"/>
@@ -2273,7 +2208,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="85" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="3"/>
       <c r="B85" s="4"/>
       <c r="C85" s="5"/>
@@ -2288,7 +2223,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="86" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="3"/>
       <c r="B86" s="4"/>
       <c r="C86" s="5"/>
@@ -2303,7 +2238,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="87" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="3"/>
       <c r="B87" s="4"/>
       <c r="C87" s="5"/>
@@ -2318,7 +2253,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="88" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="3"/>
       <c r="B88" s="4"/>
       <c r="C88" s="5"/>
@@ -2333,7 +2268,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="89" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="3"/>
       <c r="B89" s="4"/>
       <c r="C89" s="5"/>
@@ -2348,7 +2283,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="90" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="3"/>
       <c r="B90" s="4"/>
       <c r="C90" s="5"/>
@@ -2363,7 +2298,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="91" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="3"/>
       <c r="B91" s="4"/>
       <c r="C91" s="5"/>
@@ -2378,7 +2313,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="92" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="3"/>
       <c r="B92" s="4"/>
       <c r="C92" s="5"/>
@@ -2393,7 +2328,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="93" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="3"/>
       <c r="B93" s="4"/>
       <c r="C93" s="5"/>
@@ -2408,7 +2343,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="94" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="3"/>
       <c r="B94" s="4"/>
       <c r="C94" s="5"/>
@@ -2423,7 +2358,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="95" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="3"/>
       <c r="B95" s="4"/>
       <c r="C95" s="5"/>
@@ -2438,7 +2373,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="96" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="3"/>
       <c r="B96" s="4"/>
       <c r="C96" s="5"/>
@@ -2453,7 +2388,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="97" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="3"/>
       <c r="B97" s="4"/>
       <c r="C97" s="5"/>
@@ -2468,7 +2403,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="98" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="3"/>
       <c r="B98" s="4"/>
       <c r="C98" s="5"/>
@@ -2483,7 +2418,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="99" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A99" s="3"/>
       <c r="B99" s="4"/>
       <c r="C99" s="5"/>
@@ -2498,7 +2433,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="100" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="3"/>
       <c r="B100" s="4"/>
       <c r="C100" s="5"/>
@@ -2513,7 +2448,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="101" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" s="3"/>
       <c r="B101" s="4"/>
       <c r="C101" s="5"/>
@@ -2528,7 +2463,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="102" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="3"/>
       <c r="B102" s="4"/>
       <c r="C102" s="5"/>
@@ -2543,7 +2478,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="103" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="3"/>
       <c r="B103" s="4"/>
       <c r="C103" s="5"/>
@@ -2558,7 +2493,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="104" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104" s="3"/>
       <c r="B104" s="4"/>
       <c r="C104" s="5"/>
@@ -2573,7 +2508,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="105" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105" s="3"/>
       <c r="B105" s="4"/>
       <c r="C105" s="5"/>
@@ -2588,7 +2523,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="106" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A106" s="3"/>
       <c r="B106" s="4"/>
       <c r="C106" s="5"/>
@@ -2603,7 +2538,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="107" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A107" s="3"/>
       <c r="B107" s="4"/>
       <c r="C107" s="5"/>
@@ -2618,7 +2553,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="108" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A108" s="3"/>
       <c r="B108" s="4"/>
       <c r="C108" s="5"/>
@@ -2633,7 +2568,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="109" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A109" s="3"/>
       <c r="B109" s="4"/>
       <c r="C109" s="5"/>
@@ -2648,7 +2583,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="110" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A110" s="3"/>
       <c r="B110" s="4"/>
       <c r="C110" s="5"/>
@@ -2663,7 +2598,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="111" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A111" s="3"/>
       <c r="B111" s="4"/>
       <c r="C111" s="5"/>
@@ -2678,7 +2613,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="112" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A112" s="3"/>
       <c r="B112" s="4"/>
       <c r="C112" s="5"/>
@@ -2693,7 +2628,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="113" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A113" s="3"/>
       <c r="B113" s="4"/>
       <c r="C113" s="5"/>
@@ -2708,7 +2643,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="114" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A114" s="3"/>
       <c r="B114" s="4"/>
       <c r="C114" s="5"/>
@@ -2723,7 +2658,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="115" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A115" s="3"/>
       <c r="B115" s="4"/>
       <c r="C115" s="5"/>
@@ -2738,7 +2673,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="116" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A116" s="3"/>
       <c r="B116" s="4"/>
       <c r="C116" s="5"/>
@@ -2753,7 +2688,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="117" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A117" s="3"/>
       <c r="B117" s="4"/>
       <c r="C117" s="5"/>
@@ -2768,7 +2703,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="118" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A118" s="3"/>
       <c r="B118" s="4"/>
       <c r="C118" s="5"/>
@@ -2783,7 +2718,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="119" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A119" s="3"/>
       <c r="B119" s="4"/>
       <c r="C119" s="5"/>
@@ -2798,7 +2733,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="120" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A120" s="3"/>
       <c r="B120" s="4"/>
       <c r="C120" s="5"/>
@@ -2813,7 +2748,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="121" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A121" s="3"/>
       <c r="B121" s="4"/>
       <c r="C121" s="5"/>
@@ -2828,7 +2763,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="122" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A122" s="3"/>
       <c r="B122" s="4"/>
       <c r="C122" s="5"/>
@@ -2843,7 +2778,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="123" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A123" s="3"/>
       <c r="B123" s="4"/>
       <c r="C123" s="5"/>
@@ -2858,7 +2793,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="124" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A124" s="3"/>
       <c r="B124" s="4"/>
       <c r="C124" s="5"/>
@@ -2873,7 +2808,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="125" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A125" s="3"/>
       <c r="B125" s="4"/>
       <c r="C125" s="5"/>
@@ -2888,7 +2823,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="126" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A126" s="3"/>
       <c r="B126" s="4"/>
       <c r="C126" s="5"/>
@@ -2903,7 +2838,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="127" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A127" s="3"/>
       <c r="B127" s="4"/>
       <c r="C127" s="5"/>
@@ -2918,7 +2853,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="128" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A128" s="3"/>
       <c r="B128" s="4"/>
       <c r="C128" s="5"/>
@@ -2933,7 +2868,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="129" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A129" s="3"/>
       <c r="B129" s="4"/>
       <c r="C129" s="5"/>
@@ -2948,7 +2883,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="130" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A130" s="3"/>
       <c r="B130" s="4"/>
       <c r="C130" s="5"/>
@@ -2963,7 +2898,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="131" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A131" s="3"/>
       <c r="B131" s="4"/>
       <c r="C131" s="5"/>
@@ -2978,7 +2913,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="132" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A132" s="3"/>
       <c r="B132" s="4"/>
       <c r="C132" s="5"/>
@@ -2993,7 +2928,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="133" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A133" s="3"/>
       <c r="B133" s="4"/>
       <c r="C133" s="5"/>
@@ -3008,7 +2943,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="134" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A134" s="3"/>
       <c r="B134" s="4"/>
       <c r="C134" s="5"/>
@@ -3023,7 +2958,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="135" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A135" s="3"/>
       <c r="B135" s="4"/>
       <c r="C135" s="5"/>
@@ -3038,7 +2973,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="136" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A136" s="3"/>
       <c r="B136" s="4"/>
       <c r="C136" s="5"/>
@@ -3053,7 +2988,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="137" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A137" s="3"/>
       <c r="B137" s="4"/>
       <c r="C137" s="5"/>
@@ -3068,7 +3003,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="138" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A138" s="3"/>
       <c r="B138" s="4"/>
       <c r="C138" s="5"/>
@@ -3083,7 +3018,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="139" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A139" s="3"/>
       <c r="B139" s="4"/>
       <c r="C139" s="5"/>
@@ -3098,7 +3033,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="140" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A140" s="3"/>
       <c r="B140" s="4"/>
       <c r="C140" s="5"/>
@@ -3113,7 +3048,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="141" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A141" s="3"/>
       <c r="B141" s="4"/>
       <c r="C141" s="5"/>
@@ -3128,7 +3063,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="142" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A142" s="3"/>
       <c r="B142" s="4"/>
       <c r="C142" s="5"/>
@@ -3143,7 +3078,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="143" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A143" s="3"/>
       <c r="B143" s="4"/>
       <c r="C143" s="5"/>
@@ -3158,7 +3093,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="144" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A144" s="3"/>
       <c r="B144" s="4"/>
       <c r="C144" s="5"/>
@@ -3173,7 +3108,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="145" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A145" s="3"/>
       <c r="B145" s="4"/>
       <c r="C145" s="5"/>
@@ -3188,7 +3123,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="146" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A146" s="3"/>
       <c r="B146" s="4"/>
       <c r="C146" s="5"/>
@@ -3203,7 +3138,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="147" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A147" s="3"/>
       <c r="B147" s="4"/>
       <c r="C147" s="5"/>
@@ -3218,7 +3153,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="148" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A148" s="3"/>
       <c r="B148" s="4"/>
       <c r="C148" s="5"/>
@@ -3233,7 +3168,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="149" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A149" s="3"/>
       <c r="B149" s="4"/>
       <c r="C149" s="5"/>
@@ -3248,7 +3183,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="150" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A150" s="3"/>
       <c r="B150" s="4"/>
       <c r="C150" s="5"/>
@@ -3263,7 +3198,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="151" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A151" s="3"/>
       <c r="B151" s="4"/>
       <c r="C151" s="5"/>
@@ -3278,7 +3213,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="152" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A152" s="3"/>
       <c r="B152" s="4"/>
       <c r="C152" s="5"/>
@@ -3293,7 +3228,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="153" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A153" s="3"/>
       <c r="B153" s="4"/>
       <c r="C153" s="5"/>
@@ -3308,7 +3243,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="154" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A154" s="3"/>
       <c r="B154" s="4"/>
       <c r="C154" s="5"/>
@@ -3323,7 +3258,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="155" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A155" s="3"/>
       <c r="B155" s="4"/>
       <c r="C155" s="5"/>
@@ -3338,7 +3273,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="156" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A156" s="3"/>
       <c r="B156" s="4"/>
       <c r="C156" s="5"/>
@@ -3353,7 +3288,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="157" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A157" s="3"/>
       <c r="B157" s="4"/>
       <c r="C157" s="5"/>
@@ -3368,7 +3303,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="158" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A158" s="3"/>
       <c r="B158" s="4"/>
       <c r="C158" s="5"/>
@@ -3383,7 +3318,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="159" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A159" s="3"/>
       <c r="B159" s="4"/>
       <c r="C159" s="5"/>
@@ -3398,7 +3333,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="160" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A160" s="3"/>
       <c r="B160" s="4"/>
       <c r="C160" s="5"/>
@@ -3413,7 +3348,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="161" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A161" s="3"/>
       <c r="B161" s="4"/>
       <c r="C161" s="5"/>
@@ -3428,7 +3363,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="162" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A162" s="3"/>
       <c r="B162" s="4"/>
       <c r="C162" s="5"/>
@@ -3443,7 +3378,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="163" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A163" s="3"/>
       <c r="B163" s="4"/>
       <c r="C163" s="5"/>
@@ -3458,7 +3393,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="164" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A164" s="3"/>
       <c r="B164" s="4"/>
       <c r="C164" s="5"/>
@@ -3473,7 +3408,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="165" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A165" s="3"/>
       <c r="B165" s="4"/>
       <c r="C165" s="5"/>
@@ -3488,7 +3423,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="166" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A166" s="3"/>
       <c r="B166" s="4"/>
       <c r="C166" s="5"/>
@@ -3503,7 +3438,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="167" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A167" s="3"/>
       <c r="B167" s="4"/>
       <c r="C167" s="5"/>
@@ -3518,7 +3453,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="168" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A168" s="3"/>
       <c r="B168" s="4"/>
       <c r="C168" s="5"/>
@@ -3533,7 +3468,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="169" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A169" s="3"/>
       <c r="B169" s="4"/>
       <c r="C169" s="5"/>
@@ -3548,7 +3483,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="170" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A170" s="3"/>
       <c r="B170" s="4"/>
       <c r="C170" s="5"/>
@@ -3563,7 +3498,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="171" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A171" s="3"/>
       <c r="B171" s="4"/>
       <c r="C171" s="5"/>
@@ -3578,7 +3513,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="172" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A172" s="3"/>
       <c r="B172" s="4"/>
       <c r="C172" s="5"/>
@@ -3593,7 +3528,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="173" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A173" s="3"/>
       <c r="B173" s="4"/>
       <c r="C173" s="5"/>
@@ -3608,7 +3543,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="174" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A174" s="3"/>
       <c r="B174" s="4"/>
       <c r="C174" s="5"/>
@@ -3623,7 +3558,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="175" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A175" s="3"/>
       <c r="B175" s="4"/>
       <c r="C175" s="5"/>
@@ -3638,7 +3573,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="176" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A176" s="3"/>
       <c r="B176" s="4"/>
       <c r="C176" s="5"/>
@@ -3653,7 +3588,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="177" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A177" s="3"/>
       <c r="B177" s="4"/>
       <c r="C177" s="5"/>
@@ -3668,7 +3603,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="178" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A178" s="3"/>
       <c r="B178" s="4"/>
       <c r="C178" s="5"/>
@@ -3683,7 +3618,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="179" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A179" s="3"/>
       <c r="B179" s="4"/>
       <c r="C179" s="5"/>
@@ -3698,7 +3633,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="180" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A180" s="3"/>
       <c r="B180" s="4"/>
       <c r="C180" s="5"/>
@@ -3713,7 +3648,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="181" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A181" s="3"/>
       <c r="B181" s="4"/>
       <c r="C181" s="5"/>
@@ -3728,7 +3663,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="182" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A182" s="3"/>
       <c r="B182" s="4"/>
       <c r="C182" s="5"/>
@@ -3743,7 +3678,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="183" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A183" s="3"/>
       <c r="B183" s="4"/>
       <c r="C183" s="5"/>
@@ -3758,7 +3693,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="184" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A184" s="3"/>
       <c r="B184" s="4"/>
       <c r="C184" s="5"/>
@@ -3773,7 +3708,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="185" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A185" s="3"/>
       <c r="B185" s="4"/>
       <c r="C185" s="5"/>
@@ -3788,7 +3723,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="186" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A186" s="3"/>
       <c r="B186" s="4"/>
       <c r="C186" s="5"/>
@@ -3803,7 +3738,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="187" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A187" s="3"/>
       <c r="B187" s="4"/>
       <c r="C187" s="5"/>
@@ -3818,7 +3753,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="188" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A188" s="3"/>
       <c r="B188" s="4"/>
       <c r="C188" s="5"/>
@@ -3833,7 +3768,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="189" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A189" s="3"/>
       <c r="B189" s="4"/>
       <c r="C189" s="5"/>
@@ -3848,7 +3783,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="190" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A190" s="3"/>
       <c r="B190" s="4"/>
       <c r="C190" s="5"/>
@@ -3863,7 +3798,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="191" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A191" s="3"/>
       <c r="B191" s="4"/>
       <c r="C191" s="5"/>
@@ -3878,7 +3813,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="192" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A192" s="3"/>
       <c r="B192" s="4"/>
       <c r="C192" s="5"/>
@@ -3893,7 +3828,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="193" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A193" s="3"/>
       <c r="B193" s="4"/>
       <c r="C193" s="5"/>
@@ -3908,7 +3843,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="194" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A194" s="3"/>
       <c r="B194" s="4"/>
       <c r="C194" s="5"/>
@@ -3923,6 +3858,30 @@
         <v>#DIV/0!</v>
       </c>
     </row>
+    <row r="195" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A195" s="11"/>
+      <c r="B195" s="11"/>
+      <c r="C195" s="11"/>
+      <c r="D195" s="11"/>
+      <c r="E195" s="11"/>
+      <c r="F195" s="11"/>
+      <c r="G195" s="11"/>
+      <c r="H195" s="11"/>
+      <c r="I195" s="11"/>
+      <c r="J195" s="11"/>
+    </row>
+    <row r="196" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A196" s="11"/>
+      <c r="B196" s="11"/>
+      <c r="C196" s="11"/>
+      <c r="D196" s="11"/>
+      <c r="E196" s="11"/>
+      <c r="F196" s="11"/>
+      <c r="G196" s="11"/>
+      <c r="H196" s="11"/>
+      <c r="I196" s="11"/>
+      <c r="J196" s="11"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>